<commit_message>
Update Heivlinder and add Ijsvogel
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
+++ b/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
@@ -7110,7 +7110,7 @@
         <v>1</v>
       </c>
       <c r="L125" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
@@ -7186,7 +7186,7 @@
         <v>0</v>
       </c>
       <c r="L127" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.3">
@@ -7224,7 +7224,7 @@
         <v>0</v>
       </c>
       <c r="L128" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update otter en gevlekte wistnuitlibel
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
+++ b/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
@@ -3175,7 +3175,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>48</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>48</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -3289,7 +3289,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>48</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>48</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -12870,11 +12870,6 @@
     <filterColumn colId="0">
       <filters>
         <filter val="Libellen"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="nee"/>
       </filters>
     </filterColumn>
     <sortState ref="A2:L277">

</xml_diff>

<commit_message>
update witsnuitlibel en excel maatwerkgebieden
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
+++ b/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
@@ -2377,7 +2377,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2491,7 +2491,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -2681,7 +2681,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -2985,7 +2985,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -3172,7 +3172,7 @@
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -6595,7 +6595,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>230</v>
       </c>
@@ -6633,7 +6633,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>230</v>
       </c>
@@ -6671,7 +6671,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>230</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>237</v>
       </c>
@@ -6747,7 +6747,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>237</v>
       </c>
@@ -6785,7 +6785,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>237</v>
       </c>
@@ -6823,7 +6823,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>244</v>
       </c>
@@ -6861,7 +6861,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>244</v>
       </c>
@@ -6899,7 +6899,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>244</v>
       </c>
@@ -6937,7 +6937,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>244</v>
       </c>
@@ -6975,7 +6975,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>244</v>
       </c>
@@ -7013,7 +7013,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>244</v>
       </c>
@@ -7051,7 +7051,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>244</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>244</v>
       </c>
@@ -7127,7 +7127,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>244</v>
       </c>
@@ -7165,7 +7165,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>244</v>
       </c>
@@ -7203,7 +7203,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>244</v>
       </c>
@@ -7241,7 +7241,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>244</v>
       </c>
@@ -7279,7 +7279,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>244</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>244</v>
       </c>
@@ -7355,7 +7355,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>244</v>
       </c>
@@ -7393,7 +7393,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>244</v>
       </c>
@@ -7431,7 +7431,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>244</v>
       </c>
@@ -7469,7 +7469,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="136" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>244</v>
       </c>
@@ -7507,7 +7507,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>244</v>
       </c>
@@ -7545,7 +7545,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>244</v>
       </c>
@@ -7583,7 +7583,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>244</v>
       </c>
@@ -7621,7 +7621,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>244</v>
       </c>
@@ -7659,7 +7659,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>244</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>244</v>
       </c>
@@ -7735,7 +7735,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>244</v>
       </c>
@@ -7773,7 +7773,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>244</v>
       </c>
@@ -7811,7 +7811,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>244</v>
       </c>
@@ -7849,7 +7849,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>244</v>
       </c>
@@ -7887,7 +7887,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>244</v>
       </c>
@@ -7925,7 +7925,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>244</v>
       </c>
@@ -7963,7 +7963,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>244</v>
       </c>
@@ -8001,7 +8001,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>244</v>
       </c>
@@ -8039,7 +8039,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>244</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>244</v>
       </c>
@@ -8153,7 +8153,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>244</v>
       </c>
@@ -8229,7 +8229,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="156" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>244</v>
       </c>
@@ -8267,7 +8267,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="157" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>244</v>
       </c>
@@ -8343,7 +8343,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="159" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>244</v>
       </c>
@@ -8381,7 +8381,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="160" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>244</v>
       </c>
@@ -8419,7 +8419,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="161" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>244</v>
       </c>
@@ -8457,7 +8457,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="162" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>244</v>
       </c>
@@ -8495,7 +8495,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="163" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>244</v>
       </c>
@@ -8533,7 +8533,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="164" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>244</v>
       </c>
@@ -8571,7 +8571,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="165" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>244</v>
       </c>
@@ -8609,7 +8609,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="166" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>244</v>
       </c>
@@ -8647,7 +8647,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="167" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>244</v>
       </c>
@@ -8685,7 +8685,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="168" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>244</v>
       </c>
@@ -8723,7 +8723,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="169" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>244</v>
       </c>
@@ -8761,7 +8761,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="170" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>244</v>
       </c>
@@ -8799,7 +8799,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="171" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>244</v>
       </c>
@@ -8837,7 +8837,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="172" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>244</v>
       </c>
@@ -8875,7 +8875,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="173" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>244</v>
       </c>
@@ -8913,7 +8913,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="174" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>244</v>
       </c>
@@ -8951,7 +8951,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="175" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>244</v>
       </c>
@@ -8989,7 +8989,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="176" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>244</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="177" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>244</v>
       </c>
@@ -9103,7 +9103,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="179" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>363</v>
       </c>
@@ -9255,7 +9255,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="183" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>374</v>
       </c>
@@ -9293,7 +9293,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="184" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>374</v>
       </c>
@@ -9369,7 +9369,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="186" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>374</v>
       </c>
@@ -9407,7 +9407,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="187" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>374</v>
       </c>
@@ -9483,7 +9483,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="189" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>374</v>
       </c>
@@ -9521,7 +9521,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="190" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>374</v>
       </c>
@@ -9559,7 +9559,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="191" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>374</v>
       </c>
@@ -9635,7 +9635,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="193" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>374</v>
       </c>
@@ -9673,7 +9673,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="194" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>374</v>
       </c>
@@ -9711,7 +9711,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="195" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>374</v>
       </c>
@@ -9749,7 +9749,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="196" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>374</v>
       </c>
@@ -9787,7 +9787,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="197" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>374</v>
       </c>
@@ -9825,7 +9825,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="198" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>374</v>
       </c>
@@ -9863,7 +9863,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="199" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>374</v>
       </c>
@@ -9901,7 +9901,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="200" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>374</v>
       </c>
@@ -9939,7 +9939,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="201" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>374</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="202" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>374</v>
       </c>
@@ -10015,7 +10015,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="203" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>374</v>
       </c>
@@ -10053,7 +10053,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="204" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>374</v>
       </c>
@@ -10091,7 +10091,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="205" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>374</v>
       </c>
@@ -10129,7 +10129,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="206" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>374</v>
       </c>
@@ -10167,7 +10167,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="207" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>374</v>
       </c>
@@ -10205,7 +10205,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="208" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>374</v>
       </c>
@@ -10243,7 +10243,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>374</v>
       </c>
@@ -10281,7 +10281,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>374</v>
       </c>
@@ -10319,7 +10319,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>374</v>
       </c>
@@ -10357,7 +10357,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>374</v>
       </c>
@@ -10395,7 +10395,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>374</v>
       </c>
@@ -10471,7 +10471,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>374</v>
       </c>
@@ -10509,7 +10509,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>374</v>
       </c>
@@ -10547,7 +10547,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>374</v>
       </c>
@@ -10585,7 +10585,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>374</v>
       </c>
@@ -10661,7 +10661,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>374</v>
       </c>
@@ -10699,7 +10699,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>374</v>
       </c>
@@ -12181,7 +12181,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="260" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>526</v>
       </c>
@@ -12485,7 +12485,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="268" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>526</v>
       </c>
@@ -12751,7 +12751,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="275" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>526</v>
       </c>
@@ -12867,9 +12867,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L277">
-    <filterColumn colId="0">
+    <filterColumn colId="9">
       <filters>
-        <filter val="Libellen"/>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="11">
+      <filters>
+        <filter val="ja"/>
       </filters>
     </filterColumn>
     <sortState ref="A2:L277">

</xml_diff>

<commit_message>
update excel maatwerkgebieden and qgis
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
+++ b/data/input/Excel_files/Soortenlijst_Maatwerkgebieden.xlsx
@@ -2415,7 +2415,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -3137,7 +3137,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>45</v>
       </c>
@@ -5531,7 +5531,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>69</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>244</v>
       </c>
@@ -8191,7 +8191,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>244</v>
       </c>
@@ -8305,7 +8305,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="158" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>244</v>
       </c>
@@ -9445,7 +9445,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="188" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>374</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="192" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>374</v>
       </c>
@@ -10433,7 +10433,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>374</v>
       </c>
@@ -12675,7 +12675,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="273" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>526</v>
       </c>
@@ -12867,11 +12867,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L277">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="11">
       <filters>
         <filter val="ja"/>

</xml_diff>